<commit_message>
Add population age-structure pipeline and cohort-component projection model
Rebuilds pop data around single-year age/sex columns (data/pop/age), fixes
district IDs (raw dist_id was unreliable; now derived from subdist_id), and
aggregates to district/province/health-region/country levels. Adds model.ipynb
with a hybrid cohort-component projection (district rates fall back to
province rates when the historical source cohort is too small to trust) for
a 15-year population forecast. Also adds a service-volume scraper
(scrp_serv.py) and a dashboard data build script.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/data_dict-hosp.xlsx
+++ b/data/data_dict-hosp.xlsx
@@ -1607,82 +1607,82 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Include</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Index</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Source Name</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Column Name</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Column Label</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Data Type</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Unique</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Range</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Min</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Max</t>
         </is>
       </c>
-      <c r="L1" s="3" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Regex Pattern</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Default Value</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Null Value</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Format</t>
         </is>
       </c>
-      <c r="P1" s="3" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Examples</t>
         </is>
@@ -1702,7 +1702,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>str</t>
         </is>
       </c>
       <c r="G2" t="b">
@@ -1713,8 +1713,8 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Categorical with 36636 unique values: 
- [' วชิรการแพทย์คลินิก', ' ศูนย์บริการสาธารณสุข 50  บึงกุ่ม', ' โรงพยาบาลพุทธโสธร', '072 รักษา คลินิกการพยาบาลและการผดุงครรภ์', '111  คลินิกการพยาบาลและการผดุงครรภ์'] etc.</t>
+          <t>Categorical with 39454 unique values: 
+ [' วชิรการแพทย์คลินิก', ' ศูนย์บริการสาธารณสุข 50  บึงกุ่ม', '072 รักษา คลินิกการพยาบาลและการผดุงครรภ์', '111  คลินิกการพยาบาลและการผดุงครรภ์', '12 สุขดีคลินิกการพยาบาลและการผดุงครรภ์'] etc.</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -1725,8 +1725,11 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>['คลินิกรักษ์ฟัน' 'คลินิกนายแพทย์คธาวุฒิ' 'คลินิกนายแพทย์เรืองศักดิ์'
- 'คลินิกทีปวิทย์การแพทย์' 'คลินิกแพทย์นิพนธ์']</t>
+          <t>&lt;ArrowStringArray&gt;
+[           'คลินิกรักษ์ฟัน',     'คลินิกนายแพทย์คธาวุฒิ',
+ 'คลินิกนายแพทย์เรืองศักดิ์',    'คลินิกทีปวิทย์การแพทย์',
+         'คลินิกแพทย์นิพนธ์']
+Length: 5, dtype: str</t>
         </is>
       </c>
     </row>
@@ -1744,7 +1747,7 @@
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>str</t>
         </is>
       </c>
       <c r="G3" t="b">
@@ -1755,7 +1758,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Categorical with 40737 unique values: 
+          <t>Categorical with 44196 unique values: 
  ['="AA0000001"', '="AA0000002"', '="AA0000003"', '="AA0000004"', '="AA0000005"'] etc.</t>
         </is>
       </c>
@@ -1767,8 +1770,10 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t>['="CA0032045"' '="CA0032047"' '="CA0032051"' '="CA0032053"'
- '="CA0032065"']</t>
+          <t>&lt;ArrowStringArray&gt;
+['="CA0032045"', '="CA0032047"', '="CA0032051"', '="CA0032053"',
+ '="CA0032065"']
+Length: 5, dtype: str</t>
         </is>
       </c>
     </row>
@@ -1786,18 +1791,18 @@
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>str</t>
         </is>
       </c>
       <c r="G4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4" t="b">
         <v>0</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Categorical with 40726 unique values: 
+          <t>Categorical with 41207 unique values: 
  ['="000000100"', '="000000200"', '="000000300"', '="000000400"', '="000000401"'] etc.</t>
         </is>
       </c>
@@ -1809,8 +1814,10 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
-          <t>['="003204500"' '="003204700"' '="003205100"' '="003205300"'
- '="003206500"']</t>
+          <t>&lt;ArrowStringArray&gt;
+['="003204500"', '="003204700"', '="003205100"', '="003205300"',
+ '="003206500"']
+Length: 5, dtype: str</t>
         </is>
       </c>
     </row>
@@ -1828,18 +1835,18 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>str</t>
         </is>
       </c>
       <c r="G5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H5" t="b">
         <v>0</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Categorical with 40734 unique values: 
+          <t>Categorical with 41215 unique values: 
  ['="00001"', '="00002"', '="00003"', '="00004"', '="00005"'] etc.</t>
         </is>
       </c>
@@ -1851,7 +1858,9 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
-          <t>['="32045"' '="32047"' '="32051"' '="32053"' '="32065"']</t>
+          <t>&lt;ArrowStringArray&gt;
+['="32045"', '="32047"', '="32051"', '="32053"', '="32065"']
+Length: 5, dtype: str</t>
         </is>
       </c>
     </row>
@@ -1869,7 +1878,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>str</t>
         </is>
       </c>
       <c r="G6" t="b">
@@ -1880,7 +1889,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Categorical with 25808 unique values: 
+          <t>Categorical with 29235 unique values: 
  ['="           "', '=" 1010100426"', '=" ฉช-ค2/2544"', '=" ซ.8/2541"', '=" ลป-ซ1/2553"'] etc.</t>
         </is>
       </c>
@@ -1892,8 +1901,10 @@
       <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr">
         <is>
-          <t>['="30103000451"' '="30101000155"' '="30101000756"' '="30101003656"'
- '="-"']</t>
+          <t>&lt;ArrowStringArray&gt;
+['="30103000451"', '="30101000155"', '="30101000756"', '="30101003656"',
+ '="-"']
+Length: 5, dtype: str</t>
         </is>
       </c>
     </row>
@@ -1911,7 +1922,7 @@
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>str</t>
         </is>
       </c>
       <c r="G7" t="b">
@@ -1934,7 +1945,9 @@
       <c r="O7" t="inlineStr"/>
       <c r="P7" t="inlineStr">
         <is>
-          <t>['เอกชน' 'รัฐบาล']</t>
+          <t>&lt;ArrowStringArray&gt;
+['เอกชน', 'รัฐบาล']
+Length: 2, dtype: str</t>
         </is>
       </c>
     </row>
@@ -1952,7 +1965,7 @@
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>str</t>
         </is>
       </c>
       <c r="G8" t="b">
@@ -1963,7 +1976,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Categorical with 16 unique values: 
+          <t>Categorical with 17 unique values: 
  ['คลินิกเอกชน', 'ศูนย์บริการสาธารณสุข', 'ศูนย์บริการสาธารณสุข อปท.', 'ศูนย์วิชาการ', 'ศูนย์สุขภาพชุมชน ของ รพ. / เมือง (ศสม.)'] etc.</t>
         </is>
       </c>
@@ -1975,9 +1988,13 @@
       <c r="O8" t="inlineStr"/>
       <c r="P8" t="inlineStr">
         <is>
-          <t>['คลินิกเอกชน' 'โรงพยาบาลเอกชน' 'โรงพยาบาล นอก สธ.'
- 'ศูนย์สุขภาพชุมชน ของ รพ. / เมือง (ศสม.)'
- 'โรงพยาบาล/ศูนย์บริการสาธารณสุข สาขา']</t>
+          <t>&lt;ArrowStringArray&gt;
+[                            'คลินิกเอกชน',
+                          'โรงพยาบาลเอกชน',
+                       'โรงพยาบาล นอก สธ.',
+ 'ศูนย์สุขภาพชุมชน ของ รพ. / เมือง (ศสม.)',
+     'โรงพยาบาล/ศูนย์บริการสาธารณสุข สาขา']
+Length: 5, dtype: str</t>
         </is>
       </c>
     </row>
@@ -1995,11 +2012,11 @@
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>str</t>
         </is>
       </c>
       <c r="G9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H9" t="b">
         <v>0</v>
@@ -2018,8 +2035,11 @@
       <c r="O9" t="inlineStr"/>
       <c r="P9" t="inlineStr">
         <is>
-          <t>['เอกชน' 'สำนักงานศาลยุติธรรม' 'กระทรวงสาธารณสุข'
- 'องค์กรปกครองส่วนท้องถิ่น' 'กระทรวงยุติธรรม']</t>
+          <t>&lt;ArrowStringArray&gt;
+[                   'เอกชน',      'สำนักงานศาลยุติธรรม',
+         'กระทรวงสาธารณสุข', 'องค์กรปกครองส่วนท้องถิ่น',
+          'กระทรวงยุติธรรม']
+Length: 5, dtype: str</t>
         </is>
       </c>
     </row>
@@ -2037,7 +2057,7 @@
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>str</t>
         </is>
       </c>
       <c r="G10" t="b">
@@ -2060,8 +2080,11 @@
       <c r="O10" t="inlineStr"/>
       <c r="P10" t="inlineStr">
         <is>
-          <t>['-' 'สำนักงานปลัดกระทรวงสาธารณสุข' 'กรมสุขภาพจิต' 'กรมการแพทย์'
- 'กรมควบคุมโรค']</t>
+          <t>&lt;ArrowStringArray&gt;
+[                           '-', 'สำนักงานปลัดกระทรวงสาธารณสุข',
+                 'กรมสุขภาพจิต',                  'กรมการแพทย์',
+                 'กรมควบคุมโรค']
+Length: 5, dtype: str</t>
         </is>
       </c>
     </row>
@@ -2079,7 +2102,7 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>str</t>
         </is>
       </c>
       <c r="G11" t="b">
@@ -2102,9 +2125,11 @@
       <c r="O11" t="inlineStr"/>
       <c r="P11" t="inlineStr">
         <is>
-          <t>['F2 - โรงพยาบาลชุมชนขนาดกลาง' 'F1 - โรงพยาบาลชุมชนขนาดใหญ่'
- 'S - โรงพยาบาลทั่วไปขนาดใหญ่' 'F3 - โรงพยาบาลชุมชนขนาดเล็ก'
- 'M2 - โรงพยาบาลชุมชนแม่ข่าย']</t>
+          <t>&lt;ArrowStringArray&gt;
+['F2 - โรงพยาบาลชุมชนขนาดกลาง', 'F1 - โรงพยาบาลชุมชนขนาดใหญ่',
+ 'S - โรงพยาบาลทั่วไปขนาดใหญ่', 'F3 - โรงพยาบาลชุมชนขนาดเล็ก',
+  'M2 - โรงพยาบาลชุมชนแม่ข่าย']
+Length: 5, dtype: str</t>
         </is>
       </c>
     </row>
@@ -2122,7 +2147,7 @@
       <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>str</t>
         </is>
       </c>
       <c r="G12" t="b">
@@ -2145,7 +2170,9 @@
       <c r="O12" t="inlineStr"/>
       <c r="P12" t="inlineStr">
         <is>
-          <t>['ลูกข่ายภายนอกโรงพยาบาล' 'ลูกข่ายภายในโรงพยาบาล']</t>
+          <t>&lt;ArrowStringArray&gt;
+['ลูกข่ายภายนอกโรงพยาบาล', 'ลูกข่ายภายในโรงพยาบาล']
+Length: 2, dtype: str</t>
         </is>
       </c>
     </row>
@@ -2207,7 +2234,7 @@
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>str</t>
         </is>
       </c>
       <c r="G14" t="b">
@@ -2230,7 +2257,9 @@
       <c r="O14" t="inlineStr"/>
       <c r="P14" t="inlineStr">
         <is>
-          <t>['กำลังใช้งาน' 'ยกเลิก']</t>
+          <t>&lt;ArrowStringArray&gt;
+['กำลังใช้งาน', 'ยกเลิก']
+Length: 2, dtype: str</t>
         </is>
       </c>
     </row>
@@ -2248,7 +2277,7 @@
       <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>str</t>
         </is>
       </c>
       <c r="G15" t="b">
@@ -2271,8 +2300,10 @@
       <c r="O15" t="inlineStr"/>
       <c r="P15" t="inlineStr">
         <is>
-          <t>['เขตสุขภาพที่ 9' 'เขตสุขภาพที่ 6' 'เขตสุขภาพที่ 4' 'เขตสุขภาพที่ 5'
- 'เขตสุขภาพที่ 12']</t>
+          <t>&lt;ArrowStringArray&gt;
+[ 'เขตสุขภาพที่ 9',  'เขตสุขภาพที่ 6',  'เขตสุขภาพที่ 4',  'เขตสุขภาพที่ 5',
+ 'เขตสุขภาพที่ 12']
+Length: 5, dtype: str</t>
         </is>
       </c>
     </row>
@@ -2290,7 +2321,7 @@
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>str</t>
         </is>
       </c>
       <c r="G16" t="b">
@@ -2301,7 +2332,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Categorical with 22400 unique values: 
+          <t>Categorical with 24334 unique values: 
  ['(593/29-39) 591/9 ซ.สุขุมวิท 33/1 ถ.สุขุมวิท', '(๒๗๗ - ๒๗๙)', '-', '- ชั้น - ห้อง - หมู่บ้าน - ซอย - ถนน สุวรรณศร', '001 ถ.เจริญผลวัฒนา'] etc.</t>
         </is>
       </c>
@@ -2313,9 +2344,13 @@
       <c r="O16" t="inlineStr"/>
       <c r="P16" t="inlineStr">
         <is>
-          <t>['244 ถนนมิตรภาพ' '21/10 ชั้น - ห้อง - หมู่บ้าน - ซอย - ถนน -'
- '519 ถนนราษฎร์พัฒนา' '543 ชั้น - ห้อง - หมู่บ้าน - ซอย - ถนน -'
- '805 ถนนสุรนารายณ์']</t>
+          <t>&lt;ArrowStringArray&gt;
+[                            '244 ถนนมิตรภาพ',
+ '21/10 ชั้น - ห้อง - หมู่บ้าน - ซอย - ถนน -',
+                         '519 ถนนราษฎร์พัฒนา',
+   '543 ชั้น - ห้อง - หมู่บ้าน - ซอย - ถนน -',
+                          '805 ถนนสุรนารายณ์']
+Length: 5, dtype: str</t>
         </is>
       </c>
     </row>
@@ -2377,7 +2412,7 @@
       <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>str</t>
         </is>
       </c>
       <c r="G18" t="b">
@@ -2400,7 +2435,9 @@
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="inlineStr">
         <is>
-          <t>['นครราชสีมา' 'ฉะเชิงเทรา' 'ปทุมธานี' 'นนทบุรี' 'นครปฐม']</t>
+          <t>&lt;ArrowStringArray&gt;
+['นครราชสีมา', 'ฉะเชิงเทรา', 'ปทุมธานี', 'นนทบุรี', 'นครปฐม']
+Length: 5, dtype: str</t>
         </is>
       </c>
     </row>
@@ -2462,7 +2499,7 @@
       <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>str</t>
         </is>
       </c>
       <c r="G20" t="b">
@@ -2485,7 +2522,9 @@
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="inlineStr">
         <is>
-          <t>['เมืองนครราชสีมา' 'ขามทะเลสอ' 'ครบุรี' 'โนนไทย' 'ปักธงชัย']</t>
+          <t>&lt;ArrowStringArray&gt;
+['เมืองนครราชสีมา', 'ขามทะเลสอ', 'ครบุรี', 'โนนไทย', 'ปักธงชัย']
+Length: 5, dtype: str</t>
         </is>
       </c>
     </row>
@@ -2547,7 +2586,7 @@
       <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>str</t>
         </is>
       </c>
       <c r="G22" t="b">
@@ -2558,7 +2597,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Categorical with 5835 unique values: 
+          <t>Categorical with 5838 unique values: 
  ['กกกุง', 'กกดู่', 'กกตูม', 'กกทอง', 'กกปลาซิว'] etc.</t>
         </is>
       </c>
@@ -2570,7 +2609,9 @@
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="inlineStr">
         <is>
-          <t>['จอหอ' 'ขามทะเลสอ' 'แชะ' 'บ้านใหม่' 'โนนไทย']</t>
+          <t>&lt;ArrowStringArray&gt;
+['จอหอ', 'ขามทะเลสอ', 'แชะ', 'บ้านใหม่', 'โนนไทย']
+Length: 5, dtype: str</t>
         </is>
       </c>
     </row>
@@ -2588,7 +2629,7 @@
       <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>str</t>
         </is>
       </c>
       <c r="G23" t="b">
@@ -2599,8 +2640,8 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Categorical with 43 unique values: 
- ['-', '.', '0', '02', '04'] etc.</t>
+          <t>Categorical with 44 unique values: 
+ ['-', '.', '0', '01', '02'] etc.</t>
         </is>
       </c>
       <c r="J23" t="inlineStr"/>
@@ -2611,7 +2652,9 @@
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="inlineStr">
         <is>
-          <t>['3' '4' '9' '0' '14']</t>
+          <t>&lt;ArrowStringArray&gt;
+['3', '4', '9', '0', '14']
+Length: 5, dtype: str</t>
         </is>
       </c>
     </row>
@@ -2629,7 +2672,7 @@
       <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>str</t>
         </is>
       </c>
       <c r="G24" t="b">
@@ -2640,7 +2683,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Categorical with 1047 unique values: 
+          <t>Categorical with 1057 unique values: 
  ['08110', '10100', '10105', '10110', '10120'] etc.</t>
         </is>
       </c>
@@ -2652,7 +2695,9 @@
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="inlineStr">
         <is>
-          <t>['30310' '30280' '30250' '30220' '30150']</t>
+          <t>&lt;ArrowStringArray&gt;
+['30310', '30280', '30250', '30220', '30150']
+Length: 5, dtype: str</t>
         </is>
       </c>
     </row>
@@ -2670,7 +2715,7 @@
       <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>str</t>
         </is>
       </c>
       <c r="G25" t="b">
@@ -2681,8 +2726,8 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Categorical with 425 unique values: 
- [' โรงพยาบาลพุทธโสธร', 'กรมควบคุมโรค', 'กรมวิทยาศาสตร์การแพทย์', 'กองยุทธศาสตร์และแผนงาน', 'คณะทันตแพทย์ศาสตร์ มหาลัยมหิดล'] etc.</t>
+          <t>Categorical with 527 unique values: 
+ ['กรมควบคุมโรค', 'กรมวิทยาศาสตร์การแพทย์', 'กองยุทธศาสตร์และแผนงาน', 'คณะทันตแพทย์ศาสตร์  มหาวิทยาลัยเชียงใหม่', 'คณะทันตแพทย์ศาสตร์ มหาลัยมหิดล'] etc.</t>
         </is>
       </c>
       <c r="J25" t="inlineStr"/>
@@ -2693,8 +2738,13 @@
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="inlineStr">
         <is>
-          <t>['โรงพยาบาลสระบุรี' 'เทศบาลตำบลบางศรีเมือง' 'โรงพยาบาลควนเนียง'
- 'โรงพยาบาลน้ำยืน' 'โรงพยาบาลส่งเสริมสุขภาพตำบลสะเตงนอก  ตำบลสะเตงนอก']</t>
+          <t>&lt;ArrowStringArray&gt;
+[                                 'โรงพยาบาลสระบุรี',
+                             'เทศบาลตำบลบางศรีเมือง',
+                                 'โรงพยาบาลควนเนียง',
+                                   'โรงพยาบาลน้ำยืน',
+ 'โรงพยาบาลส่งเสริมสุขภาพตำบลสะเตงนอก  ตำบลสะเตงนอก']
+Length: 5, dtype: str</t>
         </is>
       </c>
     </row>
@@ -2712,7 +2762,7 @@
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>str</t>
         </is>
       </c>
       <c r="G26" t="b">
@@ -2723,8 +2773,8 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Categorical with 4481 unique values: 
- ['01/01/1954', '01/01/1957', '01/01/1972', '01/01/1974', '01/01/1982'] etc.</t>
+          <t>Categorical with 4694 unique values: 
+ ['01/01/1954', '01/01/1957', '01/01/1972', '01/01/1973', '01/01/1974'] etc.</t>
         </is>
       </c>
       <c r="J26" t="inlineStr"/>
@@ -2735,7 +2785,9 @@
       <c r="O26" t="inlineStr"/>
       <c r="P26" t="inlineStr">
         <is>
-          <t>['12/06/2017' '28/01/1952' '03/10/2011' '01/08/2020' '06/07/2017']</t>
+          <t>&lt;ArrowStringArray&gt;
+['12/06/2017', '28/01/1952', '03/10/2011', '01/08/2020', '06/07/2017']
+Length: 5, dtype: str</t>
         </is>
       </c>
     </row>
@@ -2753,7 +2805,7 @@
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>str</t>
         </is>
       </c>
       <c r="G27" t="b">
@@ -2764,7 +2816,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Categorical with 389 unique values: 
+          <t>Categorical with 429 unique values: 
  ['01/01/2014', '01/01/2015', '01/01/2019', '01/01/2020', '01/01/2023'] etc.</t>
         </is>
       </c>
@@ -2776,7 +2828,9 @@
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="inlineStr">
         <is>
-          <t>['19/02/2024' '11/09/2017' '22/09/2017' '20/06/2014' '15/02/2024']</t>
+          <t>&lt;ArrowStringArray&gt;
+['19/02/2024', '11/09/2017', '22/09/2017', '20/06/2014', '15/02/2024']
+Length: 5, dtype: str</t>
         </is>
       </c>
     </row>
@@ -2794,18 +2848,18 @@
       <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
-          <t>object</t>
+          <t>str</t>
         </is>
       </c>
       <c r="G28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H28" t="b">
         <v>0</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Categorical with 13046 unique values: 
+          <t>Categorical with 19649 unique values: 
  ['01/02/2024 02:52:33', '01/02/2024 02:59:27', '01/02/2024 03:04:31', '01/02/2024 03:08:46', '01/02/2024 03:13:09'] etc.</t>
         </is>
       </c>
@@ -2817,8 +2871,10 @@
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="inlineStr">
         <is>
-          <t>['06/10/2023 02:30:38' '06/10/2023 02:36:23' '09/10/2023 02:29:57'
- '18/11/2024 07:53:10' '21/09/2023 03:40:32']</t>
+          <t>&lt;ArrowStringArray&gt;
+['31/08/2023 06:24:29', '06/10/2023 02:30:38', '06/10/2023 02:36:23',
+ '09/10/2023 02:29:57', '18/11/2024 07:53:10']
+Length: 5, dtype: str</t>
         </is>
       </c>
     </row>

</xml_diff>